<commit_message>
the size of the tables is now a parameter of the model
</commit_message>
<xml_diff>
--- a/scripts/restaurant_variables.xlsx
+++ b/scripts/restaurant_variables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loren\Desktop\Simulation\Progetto\Restaurant_2025\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{0F366A8D-A54C-4401-A490-1D25C47DCBF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D054DCA-0056-46BE-A4A1-1143255696F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="19420" tabRatio="851" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="19420" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tables_selection" sheetId="11" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <definedName name="DatiEsterni_3" localSheetId="0" hidden="1">tables_selection!$B$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -95,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="168">
   <si>
     <t>start_timestamp</t>
   </si>
@@ -596,6 +597,9 @@
   </si>
   <si>
     <t>scenario</t>
+  </si>
+  <si>
+    <t>2_size_perc</t>
   </si>
 </sst>
 </file>
@@ -730,6 +734,21 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -908,21 +927,6 @@
     <dxf>
       <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -938,7 +942,7 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatiEsterni_3" connectionId="19" xr16:uid="{31982ACB-6682-4EA9-8905-53237B301B53}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="11" unboundColumnsLeft="1" unboundColumnsRight="3">
+  <queryTableRefresh nextId="17" unboundColumnsLeft="1" unboundColumnsRight="3">
     <queryTableFields count="10">
       <queryTableField id="10" dataBound="0" tableColumnId="10"/>
       <queryTableField id="1" name="start_timestamp" tableColumnId="1"/>
@@ -979,10 +983,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7D1585E5-EB18-4555-BFB4-AB049789BB50}" name="tables_selection" displayName="tables_selection" ref="A1:J11" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:J11" xr:uid="{7D1585E5-EB18-4555-BFB4-AB049789BB50}"/>
   <tableColumns count="10">
-    <tableColumn id="10" xr3:uid="{1ADF8E6C-C756-4DB0-AF29-730090E9A389}" uniqueName="10" name="scenario" queryTableFieldId="10" dataDxfId="19"/>
-    <tableColumn id="1" xr3:uid="{9DF6AF6D-4327-4E8B-A17C-4CE32200A2CC}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{DB186560-5030-4DB1-A6BD-A74C44B2F90A}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{6CE09762-A225-468B-8C15-326E109C4C41}" uniqueName="3" name="period" queryTableFieldId="3" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{1ADF8E6C-C756-4DB0-AF29-730090E9A389}" uniqueName="10" name="scenario" queryTableFieldId="10" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{9DF6AF6D-4327-4E8B-A17C-4CE32200A2CC}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{DB186560-5030-4DB1-A6BD-A74C44B2F90A}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{6CE09762-A225-468B-8C15-326E109C4C41}" uniqueName="3" name="period" queryTableFieldId="3" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{90771DE1-93AE-42DD-88DE-8292168CC27F}" uniqueName="4" name="bar_on" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{2D6F5E1B-E207-46D0-A78B-EA6977317860}" uniqueName="5" name="inside_on" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{5AFB94CB-8BB6-4AE5-B6B3-D1BD6C86A1FB}" uniqueName="6" name="outside_on" queryTableFieldId="6"/>
@@ -998,12 +1002,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{54D2211C-274A-47E4-BDD0-4C0951D8DD68}" name="employees_schedule" displayName="employees_schedule" ref="A1:H71" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H71" xr:uid="{54D2211C-274A-47E4-BDD0-4C0951D8DD68}"/>
   <tableColumns count="8">
-    <tableColumn id="15" xr3:uid="{C7ED7AB4-5A31-4D81-834A-B6E64F7023C8}" uniqueName="15" name="scenario" queryTableFieldId="9" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{1826F0BC-F6D0-44C5-8A93-C7D99BD8CB8B}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{75D23335-1496-4011-81D1-D6034B72FF11}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{92C90E84-B1B0-4866-9DDC-2A2B72F890FA}" uniqueName="4" name="weekday" queryTableFieldId="4" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{954429F6-A3DE-46A7-885B-49BC6CAF5664}" uniqueName="5" name="hour" queryTableFieldId="5" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{D0D42E6A-14B4-4741-A3F6-DD9143A88038}" uniqueName="6" name="period" queryTableFieldId="6" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{C7ED7AB4-5A31-4D81-834A-B6E64F7023C8}" uniqueName="15" name="scenario" queryTableFieldId="9" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{1826F0BC-F6D0-44C5-8A93-C7D99BD8CB8B}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{75D23335-1496-4011-81D1-D6034B72FF11}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{92C90E84-B1B0-4866-9DDC-2A2B72F890FA}" uniqueName="4" name="weekday" queryTableFieldId="4" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{954429F6-A3DE-46A7-885B-49BC6CAF5664}" uniqueName="5" name="hour" queryTableFieldId="5" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{D0D42E6A-14B4-4741-A3F6-DD9143A88038}" uniqueName="6" name="period" queryTableFieldId="6" dataDxfId="15"/>
     <tableColumn id="7" xr3:uid="{DC0D317B-9907-4E39-BD04-56F982B6DFC4}" uniqueName="7" name="waiters" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{5822B03F-BA67-4CAF-8288-1B9FA740A60F}" uniqueName="8" name="cooks" queryTableFieldId="8"/>
   </tableColumns>
@@ -1012,14 +1016,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}" name="Tabella3" displayName="Tabella3" ref="A1:E11" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}" name="Tabella3" displayName="Tabella3" ref="A1:E11" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
   <autoFilter ref="A1:E11" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5F6DE45A-D069-49C3-A965-E57C526C9F10}" name="scenario" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{4D8F0B29-A4FF-499D-9A3B-DCD79E56771F}" name="start_timestamp" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{73FD92A6-7E32-4F59-A6D2-E391CC1529B2}" name="end_timestamp" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{E9B6B43D-80B9-448F-8CE5-DB0428CE9192}" name="period" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{FA561D75-B96F-4DC4-B290-98BCE5AF9EBB}" name="time_avg" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5F6DE45A-D069-49C3-A965-E57C526C9F10}" name="scenario" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{4D8F0B29-A4FF-499D-9A3B-DCD79E56771F}" name="start_timestamp" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{73FD92A6-7E32-4F59-A6D2-E391CC1529B2}" name="end_timestamp" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{E9B6B43D-80B9-448F-8CE5-DB0428CE9192}" name="period" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{FA561D75-B96F-4DC4-B290-98BCE5AF9EBB}" name="time_avg" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1032,7 +1036,7 @@
     <tableColumn id="1" xr3:uid="{C0C152CA-AC82-4A38-9515-01F93B55CD35}" name="scenario"/>
     <tableColumn id="2" xr3:uid="{A9274257-0F1F-4EC5-AEAD-2D02ED20F27D}" name="start_timestamp"/>
     <tableColumn id="3" xr3:uid="{8EBF5A3E-33DA-4E63-85B2-6A750FD2B59E}" name="end_timestamp"/>
-    <tableColumn id="4" xr3:uid="{1B570803-0CC6-4039-83E4-466D06E97DE8}" name="arrival_rate" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{1B570803-0CC6-4039-83E4-466D06E97DE8}" name="arrival_rate" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{2330BE18-97F9-494B-A0D2-BC6CD4BE5D26}" name="weekday"/>
     <tableColumn id="6" xr3:uid="{511C9B76-5714-4C6E-B45F-24A76465D0A2}" name="hour"/>
     <tableColumn id="7" xr3:uid="{DDB83C9A-5515-4339-958C-0504A36D7FBA}" name="avg_group_size"/>
@@ -1304,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2489A5EA-DD05-4EB8-ADF0-37ED0B27C5D1}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.26953125" style="3" bestFit="1" customWidth="1"/>
@@ -1314,7 +1318,10 @@
     <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.54296875" style="3" customWidth="1"/>
+    <col min="12" max="14" width="12.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
changed visualization of pml model
</commit_message>
<xml_diff>
--- a/scripts/restaurant_variables.xlsx
+++ b/scripts/restaurant_variables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loren\Desktop\Simulation\Progetto\Restaurant_2025\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6389F4E-875A-48A8-9645-FAEAFE40CB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FF148C4-FB29-4439-BB2F-CFB750259F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="19420" tabRatio="851" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -744,6 +744,15 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="23">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -908,6 +917,18 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
@@ -921,27 +942,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -999,10 +999,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7D1585E5-EB18-4555-BFB4-AB049789BB50}" name="tables_selection" displayName="tables_selection" ref="A1:J11" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:J11" xr:uid="{7D1585E5-EB18-4555-BFB4-AB049789BB50}"/>
   <tableColumns count="10">
-    <tableColumn id="10" xr3:uid="{1ADF8E6C-C756-4DB0-AF29-730090E9A389}" uniqueName="10" name="scenario" queryTableFieldId="10" dataDxfId="19"/>
-    <tableColumn id="1" xr3:uid="{9DF6AF6D-4327-4E8B-A17C-4CE32200A2CC}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{DB186560-5030-4DB1-A6BD-A74C44B2F90A}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{6CE09762-A225-468B-8C15-326E109C4C41}" uniqueName="3" name="period" queryTableFieldId="3" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{1ADF8E6C-C756-4DB0-AF29-730090E9A389}" uniqueName="10" name="scenario" queryTableFieldId="10" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{9DF6AF6D-4327-4E8B-A17C-4CE32200A2CC}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{DB186560-5030-4DB1-A6BD-A74C44B2F90A}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{6CE09762-A225-468B-8C15-326E109C4C41}" uniqueName="3" name="period" queryTableFieldId="3" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{90771DE1-93AE-42DD-88DE-8292168CC27F}" uniqueName="4" name="bar_on" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{2D6F5E1B-E207-46D0-A78B-EA6977317860}" uniqueName="5" name="inside_on" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{5AFB94CB-8BB6-4AE5-B6B3-D1BD6C86A1FB}" uniqueName="6" name="outside_on" queryTableFieldId="6"/>
@@ -1018,12 +1018,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{54D2211C-274A-47E4-BDD0-4C0951D8DD68}" name="employees_schedule" displayName="employees_schedule" ref="A1:H71" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H71" xr:uid="{54D2211C-274A-47E4-BDD0-4C0951D8DD68}"/>
   <tableColumns count="8">
-    <tableColumn id="15" xr3:uid="{C7ED7AB4-5A31-4D81-834A-B6E64F7023C8}" uniqueName="15" name="scenario" queryTableFieldId="9" dataDxfId="15"/>
-    <tableColumn id="1" xr3:uid="{1826F0BC-F6D0-44C5-8A93-C7D99BD8CB8B}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{75D23335-1496-4011-81D1-D6034B72FF11}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{92C90E84-B1B0-4866-9DDC-2A2B72F890FA}" uniqueName="4" name="weekday" queryTableFieldId="4" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{954429F6-A3DE-46A7-885B-49BC6CAF5664}" uniqueName="5" name="hour" queryTableFieldId="5" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{D0D42E6A-14B4-4741-A3F6-DD9143A88038}" uniqueName="6" name="period" queryTableFieldId="6" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{C7ED7AB4-5A31-4D81-834A-B6E64F7023C8}" uniqueName="15" name="scenario" queryTableFieldId="9" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{1826F0BC-F6D0-44C5-8A93-C7D99BD8CB8B}" uniqueName="1" name="start_timestamp" queryTableFieldId="1" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{75D23335-1496-4011-81D1-D6034B72FF11}" uniqueName="2" name="end_timestamp" queryTableFieldId="2" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{92C90E84-B1B0-4866-9DDC-2A2B72F890FA}" uniqueName="4" name="weekday" queryTableFieldId="4" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{954429F6-A3DE-46A7-885B-49BC6CAF5664}" uniqueName="5" name="hour" queryTableFieldId="5" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{D0D42E6A-14B4-4741-A3F6-DD9143A88038}" uniqueName="6" name="period" queryTableFieldId="6" dataDxfId="17"/>
     <tableColumn id="7" xr3:uid="{DC0D317B-9907-4E39-BD04-56F982B6DFC4}" uniqueName="7" name="waiters" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{5822B03F-BA67-4CAF-8288-1B9FA740A60F}" uniqueName="8" name="cooks" queryTableFieldId="8"/>
   </tableColumns>
@@ -1032,14 +1032,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}" name="Tabella3" displayName="Tabella3" ref="A1:E11" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}" name="Tabella3" displayName="Tabella3" ref="A1:E11" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:E11" xr:uid="{D544813D-DF99-41C8-AE8A-38BE1FAF9E94}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{5F6DE45A-D069-49C3-A965-E57C526C9F10}" name="scenario" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{4D8F0B29-A4FF-499D-9A3B-DCD79E56771F}" name="start_timestamp" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{73FD92A6-7E32-4F59-A6D2-E391CC1529B2}" name="end_timestamp" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{E9B6B43D-80B9-448F-8CE5-DB0428CE9192}" name="period" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{FA561D75-B96F-4DC4-B290-98BCE5AF9EBB}" name="time_avg" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5F6DE45A-D069-49C3-A965-E57C526C9F10}" name="scenario" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{4D8F0B29-A4FF-499D-9A3B-DCD79E56771F}" name="start_timestamp" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{73FD92A6-7E32-4F59-A6D2-E391CC1529B2}" name="end_timestamp" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{E9B6B43D-80B9-448F-8CE5-DB0428CE9192}" name="period" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{FA561D75-B96F-4DC4-B290-98BCE5AF9EBB}" name="time_avg" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1050,9 +1050,9 @@
   <autoFilter ref="A1:G239" xr:uid="{E79869A8-51C0-465F-A154-CE9C9BB79619}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C0C152CA-AC82-4A38-9515-01F93B55CD35}" name="scenario"/>
-    <tableColumn id="2" xr3:uid="{A9274257-0F1F-4EC5-AEAD-2D02ED20F27D}" name="start_timestamp" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{8EBF5A3E-33DA-4E63-85B2-6A750FD2B59E}" name="end_timestamp" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{1B570803-0CC6-4039-83E4-466D06E97DE8}" name="arrival_rate" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{A9274257-0F1F-4EC5-AEAD-2D02ED20F27D}" name="start_timestamp" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{8EBF5A3E-33DA-4E63-85B2-6A750FD2B59E}" name="end_timestamp" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{1B570803-0CC6-4039-83E4-466D06E97DE8}" name="arrival_rate" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{2330BE18-97F9-494B-A0D2-BC6CD4BE5D26}" name="weekday"/>
     <tableColumn id="6" xr3:uid="{511C9B76-5714-4C6E-B45F-24A76465D0A2}" name="hour"/>
     <tableColumn id="7" xr3:uid="{DDB83C9A-5515-4339-958C-0504A36D7FBA}" name="avg_group_size"/>
@@ -2385,10 +2385,10 @@
         <v>158</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -2515,10 +2515,10 @@
         <v>158</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -2645,10 +2645,10 @@
         <v>158</v>
       </c>
       <c r="G36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H36">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>